<commit_message>
Replace report.xlsx new update til solution2
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\22972\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C664991-BDDD-4499-8C62-453941567590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A3B406-FAE4-4126-8A7D-D3E2191EF675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1588,14 +1588,16 @@
       <c r="C23" s="8">
         <v>20</v>
       </c>
-      <c r="D23" s="7"/>
+      <c r="D23" s="12">
+        <v>1</v>
+      </c>
       <c r="E23" s="7"/>
       <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
       <c r="I23" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1609,13 +1611,15 @@
         <v>15</v>
       </c>
       <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
+      <c r="E24" s="12">
+        <v>1</v>
+      </c>
       <c r="F24" s="7"/>
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
       <c r="I24" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -1630,12 +1634,14 @@
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
+      <c r="F25" s="12">
+        <v>1</v>
+      </c>
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
       <c r="I25" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1648,14 +1654,16 @@
       <c r="C26" s="8">
         <v>5</v>
       </c>
-      <c r="D26" s="7"/>
+      <c r="D26" s="12">
+        <v>1</v>
+      </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
       <c r="I26" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1668,14 +1676,16 @@
       <c r="C27" s="8">
         <v>5</v>
       </c>
-      <c r="D27" s="7"/>
+      <c r="D27" s="12">
+        <v>1</v>
+      </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
       <c r="I27" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -1691,11 +1701,13 @@
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
       <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
+      <c r="G28" s="12">
+        <v>1</v>
+      </c>
       <c r="H28" s="7"/>
       <c r="I28" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -1711,11 +1723,13 @@
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
+      <c r="G29" s="12">
+        <v>1</v>
+      </c>
       <c r="H29" s="7"/>
       <c r="I29" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -1728,14 +1742,16 @@
       <c r="C30" s="8">
         <v>15</v>
       </c>
-      <c r="D30" s="7"/>
+      <c r="D30" s="12">
+        <v>1</v>
+      </c>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
       <c r="I30" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1751,11 +1767,13 @@
       <c r="D31" s="7"/>
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
+      <c r="G31" s="12">
+        <v>1</v>
+      </c>
       <c r="H31" s="7"/>
       <c r="I31" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -1770,12 +1788,14 @@
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
+      <c r="F32" s="12">
+        <v>1</v>
+      </c>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
       <c r="I32" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -1790,12 +1810,14 @@
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
+      <c r="F33" s="12">
+        <v>1</v>
+      </c>
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
       <c r="I33" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -1809,13 +1831,15 @@
         <v>30</v>
       </c>
       <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
+      <c r="E34" s="12">
+        <v>1</v>
+      </c>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
       <c r="H34" s="7"/>
       <c r="I34" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -1829,19 +1853,19 @@
       </c>
       <c r="D35">
         <f>SUMPRODUCT(D23:D34,$C23:$C34)</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="E35">
         <f t="shared" ref="E35:H35" si="3">SUMPRODUCT(E23:E34,$C23:$C34)</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F35">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G35">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="H35">
         <f t="shared" si="3"/>
@@ -1850,7 +1874,7 @@
       <c r="I35" s="1"/>
       <c r="K35">
         <f>SUM(D35:H35)</f>
-        <v>0</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Replace report.xlsx GOR inserted
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\22972\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24A3B406-FAE4-4126-8A7D-D3E2191EF675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{327B2B3B-D067-4567-A8B8-FDAAF432AF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2054,14 +2054,16 @@
       <c r="B46" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D46" s="7"/>
+      <c r="D46" s="12"/>
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
+      <c r="G46" s="12">
+        <v>1</v>
+      </c>
       <c r="H46" s="7"/>
       <c r="I46" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -2071,14 +2073,16 @@
       <c r="B47" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="D47" s="7"/>
+      <c r="D47" s="12">
+        <v>1</v>
+      </c>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
       <c r="H47" s="7"/>
       <c r="I47" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -2088,14 +2092,16 @@
       <c r="B48" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D48" s="7"/>
+      <c r="D48" s="12">
+        <v>1</v>
+      </c>
       <c r="E48" s="7"/>
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
       <c r="H48" s="7"/>
       <c r="I48" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -2105,14 +2111,16 @@
       <c r="B49" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D49" s="7"/>
+      <c r="D49" s="12">
+        <v>1</v>
+      </c>
       <c r="E49" s="7"/>
       <c r="F49" s="7"/>
       <c r="G49" s="7"/>
       <c r="H49" s="7"/>
       <c r="I49" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -2125,11 +2133,13 @@
       <c r="D50" s="7"/>
       <c r="E50" s="7"/>
       <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
+      <c r="G50" s="12">
+        <v>1</v>
+      </c>
       <c r="H50" s="7"/>
       <c r="I50" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -2207,14 +2217,16 @@
       <c r="B55" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="D55" s="7"/>
+      <c r="D55" s="12">
+        <v>1</v>
+      </c>
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
       <c r="G55" s="7"/>
       <c r="H55" s="7"/>
       <c r="I55" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -2224,14 +2236,16 @@
       <c r="B56" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D56" s="7"/>
+      <c r="D56" s="12"/>
       <c r="E56" s="7"/>
       <c r="F56" s="7"/>
-      <c r="G56" s="7"/>
+      <c r="G56" s="12">
+        <v>1</v>
+      </c>
       <c r="H56" s="7"/>
       <c r="I56" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
@@ -2241,14 +2255,18 @@
       <c r="B57" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D57" s="7"/>
+      <c r="D57" s="12">
+        <v>0.3</v>
+      </c>
       <c r="E57" s="7"/>
       <c r="F57" s="7"/>
-      <c r="G57" s="7"/>
+      <c r="G57" s="12">
+        <v>0.7</v>
+      </c>
       <c r="H57" s="7"/>
       <c r="I57" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
@@ -2258,14 +2276,16 @@
       <c r="B58" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D58" s="7"/>
+      <c r="D58" s="12">
+        <v>1</v>
+      </c>
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
       <c r="G58" s="7"/>
       <c r="H58" s="7"/>
       <c r="I58" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
@@ -2275,14 +2295,16 @@
       <c r="B59" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="D59" s="7"/>
+      <c r="D59" s="12">
+        <v>1</v>
+      </c>
       <c r="E59" s="7"/>
       <c r="F59" s="7"/>
       <c r="G59" s="7"/>
       <c r="H59" s="7"/>
       <c r="I59" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
@@ -2292,14 +2314,16 @@
       <c r="B60" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D60" s="7"/>
+      <c r="D60" s="12">
+        <v>0.7</v>
+      </c>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
       <c r="G60" s="7"/>
       <c r="H60" s="7"/>
       <c r="I60" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>70%</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
@@ -2326,14 +2350,18 @@
       <c r="B62" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D62" s="7"/>
+      <c r="D62" s="12">
+        <v>0.2</v>
+      </c>
       <c r="E62" s="7"/>
       <c r="F62" s="7"/>
-      <c r="G62" s="7"/>
+      <c r="G62" s="12">
+        <v>0.8</v>
+      </c>
       <c r="H62" s="7"/>
       <c r="I62" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -2346,11 +2374,13 @@
       <c r="D63" s="7"/>
       <c r="E63" s="7"/>
       <c r="F63" s="7"/>
-      <c r="G63" s="7"/>
+      <c r="G63" s="12">
+        <v>1</v>
+      </c>
       <c r="H63" s="7"/>
       <c r="I63" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -2360,21 +2390,23 @@
       <c r="B64" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="D64" s="7"/>
+      <c r="D64" s="12">
+        <v>1</v>
+      </c>
       <c r="E64" s="7"/>
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
       <c r="H64" s="7"/>
       <c r="I64" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>0%</v>
+        <v>100%</v>
       </c>
     </row>
     <row r="65" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C65" s="8"/>
       <c r="D65">
         <f t="shared" ref="D65:G65" si="5">SUM(D36:D64)</f>
-        <v>0</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="E65">
         <f t="shared" si="5"/>
@@ -2386,7 +2418,7 @@
       </c>
       <c r="G65">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="H65">
         <f>SUM(H36:H64)</f>
@@ -2394,7 +2426,7 @@
       </c>
       <c r="K65">
         <f>SUM(D65:H65)</f>
-        <v>0</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="67" spans="3:11" x14ac:dyDescent="0.25">

</xml_diff>